<commit_message>
chose to omit talkstepfather and talkstepmother
</commit_message>
<xml_diff>
--- a/HBSC_data/hbsc_variable_groupings.xlsx
+++ b/HBSC_data/hbsc_variable_groupings.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fongkangwei/nus/ay25_26/sem2/DSA4262/dsa4262-group-3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fongkangwei/nus/ay25_26/sem2/DSA4262/dsa4262-group-3/HBSC_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FE694FA-AC71-6D40-83A5-36F303D06571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D73BF91A-94B2-BB44-A658-078A2DFAFF84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-6980" yWindow="-28800" windowWidth="51200" windowHeight="28800" xr2:uid="{3AF0AE97-7F91-F64F-88C9-E497DF8BD89E}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17340" xr2:uid="{3AF0AE97-7F91-F64F-88C9-E497DF8BD89E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="160">
   <si>
     <t>new question</t>
   </si>
@@ -514,16 +514,7 @@
     <t>talk father</t>
   </si>
   <si>
-    <t>How easy is it for you to talk to your father/stepfather about things that really bother you?</t>
-  </si>
-  <si>
-    <t>take the column that has value 1-4. if both have 1-4, then take mean of both values</t>
-  </si>
-  <si>
     <t>talk mother</t>
-  </si>
-  <si>
-    <t>How easy is it for you to talk to your mother/stepmother about things that really bother you?</t>
   </si>
   <si>
     <t>fam sup</t>
@@ -2151,12 +2142,6 @@
       <c r="B109" t="s">
         <v>156</v>
       </c>
-      <c r="C109" t="s">
-        <v>158</v>
-      </c>
-      <c r="D109" t="s">
-        <v>157</v>
-      </c>
       <c r="E109" t="s">
         <v>124</v>
       </c>
@@ -2168,14 +2153,8 @@
       <c r="A110" t="s">
         <v>111</v>
       </c>
-      <c r="B110" t="s">
-        <v>156</v>
-      </c>
       <c r="E110" t="s">
-        <v>124</v>
-      </c>
-      <c r="F110" t="s">
-        <v>124</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.2">
@@ -2183,13 +2162,7 @@
         <v>112</v>
       </c>
       <c r="B111" t="s">
-        <v>159</v>
-      </c>
-      <c r="C111" t="s">
-        <v>158</v>
-      </c>
-      <c r="D111" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E111" t="s">
         <v>124</v>
@@ -2202,14 +2175,8 @@
       <c r="A112" t="s">
         <v>113</v>
       </c>
-      <c r="B112" t="s">
-        <v>159</v>
-      </c>
       <c r="E112" t="s">
-        <v>124</v>
-      </c>
-      <c r="F112" t="s">
-        <v>124</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.2">
@@ -2228,13 +2195,13 @@
         <v>115</v>
       </c>
       <c r="B114" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C114" t="s">
         <v>136</v>
       </c>
       <c r="D114" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E114" t="s">
         <v>124</v>
@@ -2248,7 +2215,7 @@
         <v>116</v>
       </c>
       <c r="B115" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="E115" t="s">
         <v>124</v>

</xml_diff>

<commit_message>
Replace main with latest local prototype
</commit_message>
<xml_diff>
--- a/HBSC_data/hbsc_variable_groupings.xlsx
+++ b/HBSC_data/hbsc_variable_groupings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fongkangwei/nus/ay25_26/sem2/DSA4262/dsa4262-group-3/HBSC_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D73BF91A-94B2-BB44-A658-078A2DFAFF84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35B531AB-8B54-3343-A764-7735EAEBBE1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17340" xr2:uid="{3AF0AE97-7F91-F64F-88C9-E497DF8BD89E}"/>
+    <workbookView xWindow="0" yWindow="1780" windowWidth="29400" windowHeight="17340" xr2:uid="{3AF0AE97-7F91-F64F-88C9-E497DF8BD89E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="157">
   <si>
     <t>new question</t>
   </si>
@@ -47,9 +47,6 @@
     <t>Y</t>
   </si>
   <si>
-    <t>HBSC', 'seqno_int', 'cluster', 'countryno', 'region', 'id1', 'id2', 'id3', 'id4', 'weight', 'adm', 'month', 'year', 'age', 'agecat', 'sex', 'grade', 'monthbirth', 'yearbirth', 'fasfamcar', 'fasbedroom', 'fascomputers', 'fasbathroom', 'fasdishwash', 'fasholidays', 'health', 'lifesat', 'headache', 'stomachache', 'backache', 'feellow', 'irritable', 'nervous', 'sleepdificulty', 'dizzy', 'thinkbody', 'physact60', 'breakfastwd', 'breakfastwe', 'fruits_2', 'vegetables_2', 'sweets_2', 'softdrinks_2', 'fmeal', 'toothbr', 'timeexe', 'smokltm', 'smok30d_2', 'alcltm', 'alc30d_2', 'drunkltm', 'drunk30d', 'cannabisltm_2', 'cannabis30d_2', 'bodyweight', 'bodyheight', 'likeschool', 'schoolpressure', 'studtogether', 'studhelpful', 'studaccept', 'teacheraccept', 'teachercare', 'teachertrust', 'bulliedothers', 'beenbullied', 'cbulliedothers', 'cbeenbullied', 'fight12m', 'injured12m', 'friendhelp', 'friendcounton', 'friendshare', 'friendtalk', 'emconlfreq1', 'emconlfreq2', 'emconlfreq3', 'emconlfreq4', 'emconlpref1', 'emconlpref2', 'emconlpref3', 'emcsocmed1', 'emcsocmed2', 'emcsocmed3', 'emcsocmed4', 'emcsocmed5', 'emcsocmed6', 'emcsocmed7', 'emcsocmed8', 'emcsocmed9', 'hadsex', 'agesex', 'contraceptcondom', 'contraceptpill', 'countryborn', 'countrybornmo', 'countrybornfa', 'motherhome1', 'fatherhome1', 'stepmohome1', 'stepfahome1', 'fosterhome1', 'elsehome1_2', 'employfa', 'employmo', 'employnotfa', 'employnotmo', 'talkfather', 'talkstepfa', 'talkmother', 'talkstepmo', 'famhelp', 'famsup', 'famtalk', 'famdec', 'MBMI', 'IRFAS', 'IRRELFAS_LMH', 'IOTF4', 'oweight_who'</t>
-  </si>
-  <si>
     <t>HBSC'</t>
   </si>
   <si>
@@ -465,9 +462,6 @@
   </si>
   <si>
     <t>teacher</t>
-  </si>
-  <si>
-    <t>I feel that my teachers care about and accept me.</t>
   </si>
   <si>
     <t>bully others</t>
@@ -511,16 +505,13 @@
     <t>else home</t>
   </si>
   <si>
-    <t>talk father</t>
-  </si>
-  <si>
-    <t>talk mother</t>
-  </si>
-  <si>
     <t>fam sup</t>
   </si>
   <si>
     <t>I get the emotional help and support I need (eg. talking about my problems) from my family.</t>
+  </si>
+  <si>
+    <t>I feel that my teachers care about and accept me as I am.</t>
   </si>
 </sst>
 </file>
@@ -902,159 +893,154 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DB3725F-D3FC-2E47-A8B6-31ABFEEC6E95}">
-  <dimension ref="A1:BJ121"/>
+  <dimension ref="A1:F121"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="13.1640625" customWidth="1"/>
-    <col min="3" max="3" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="46" customWidth="1"/>
     <col min="4" max="4" width="94.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D1" t="s">
         <v>0</v>
       </c>
       <c r="E1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="2" spans="1:62" x14ac:dyDescent="0.2">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="E2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="E3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="E3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="E4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="E4" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="E5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="E5" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="E6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="E6" t="s">
-        <v>1</v>
-      </c>
-      <c r="H6" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="E7" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>8</v>
       </c>
-      <c r="E7" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="E8" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>9</v>
       </c>
-      <c r="E8" t="s">
-        <v>1</v>
-      </c>
-      <c r="BJ8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="E9" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>10</v>
       </c>
-      <c r="E9" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="E10" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>11</v>
       </c>
-      <c r="E10" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="E11" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
         <v>12</v>
       </c>
-      <c r="E11" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="E12" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>13</v>
       </c>
-      <c r="E12" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+      <c r="E13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="E13" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="E14" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>15</v>
       </c>
-      <c r="E14" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+      <c r="E15" t="s">
+        <v>123</v>
+      </c>
+      <c r="F15" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>16</v>
-      </c>
-      <c r="E15" t="s">
-        <v>124</v>
-      </c>
-      <c r="F15" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:62" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>17</v>
       </c>
       <c r="E16" t="s">
         <v>1</v>
@@ -1062,10 +1048,10 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E17" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F17" t="s">
         <v>1</v>
@@ -1073,7 +1059,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E18" t="s">
         <v>1</v>
@@ -1081,7 +1067,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E19" t="s">
         <v>1</v>
@@ -1089,7 +1075,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E20" t="s">
         <v>1</v>
@@ -1097,10 +1083,10 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E21" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F21" t="s">
         <v>1</v>
@@ -1108,10 +1094,10 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E22" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F22" t="s">
         <v>1</v>
@@ -1119,10 +1105,10 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E23" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F23" t="s">
         <v>1</v>
@@ -1130,10 +1116,10 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E24" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F24" t="s">
         <v>1</v>
@@ -1141,10 +1127,10 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E25" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F25" t="s">
         <v>1</v>
@@ -1152,10 +1138,10 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E26" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F26" t="s">
         <v>1</v>
@@ -1163,18 +1149,18 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E27" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F27" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E28" t="s">
         <v>1</v>
@@ -1182,55 +1168,55 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B29" t="s">
+        <v>126</v>
+      </c>
+      <c r="C29" t="s">
+        <v>130</v>
+      </c>
+      <c r="D29" t="s">
         <v>127</v>
       </c>
-      <c r="C29" t="s">
-        <v>131</v>
-      </c>
-      <c r="D29" t="s">
-        <v>128</v>
-      </c>
       <c r="E29" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F29" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B30" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E30" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F30" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B31" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E32" t="s">
         <v>1</v>
@@ -1238,7 +1224,7 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E33" t="s">
         <v>1</v>
@@ -1246,7 +1232,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E34" t="s">
         <v>1</v>
@@ -1254,189 +1240,189 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E35" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F35" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B36" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E37" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F37" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E38" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F38" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B39" t="s">
+        <v>132</v>
+      </c>
+      <c r="C39" t="s">
         <v>133</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>134</v>
       </c>
-      <c r="D39" t="s">
-        <v>135</v>
-      </c>
       <c r="E39" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F39" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B40" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E40" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F40" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B41" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C41" t="s">
+        <v>135</v>
+      </c>
+      <c r="D41" t="s">
         <v>136</v>
       </c>
-      <c r="D41" t="s">
-        <v>137</v>
-      </c>
       <c r="E41" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F41" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B42" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B43" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C43" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D43" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E43" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F43" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B44" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E44" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F44" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E45" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F45" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E46" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F46" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E47" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F47" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E48" t="s">
         <v>1</v>
@@ -1444,7 +1430,7 @@
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E49" t="s">
         <v>1</v>
@@ -1452,7 +1438,7 @@
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E50" t="s">
         <v>1</v>
@@ -1460,7 +1446,7 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E51" t="s">
         <v>1</v>
@@ -1468,7 +1454,7 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E52" t="s">
         <v>1</v>
@@ -1476,7 +1462,7 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E53" t="s">
         <v>1</v>
@@ -1484,7 +1470,7 @@
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E54" t="s">
         <v>1</v>
@@ -1492,7 +1478,7 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E55" t="s">
         <v>1</v>
@@ -1500,10 +1486,10 @@
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E56" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F56" t="s">
         <v>1</v>
@@ -1511,10 +1497,10 @@
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E57" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F57" t="s">
         <v>1</v>
@@ -1522,301 +1508,301 @@
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E58" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F58" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E59" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F59" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E60" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F60" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E61" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F61" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E62" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F62" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B63" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C63" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D63" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="E63" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F63" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B64" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E64" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F64" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E65" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F65" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B66" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C66" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D66" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E66" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F66" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B67" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C67" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D67" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E67" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F67" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B68" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E68" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F68" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B69" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E69" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F69" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E70" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F70" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E71" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F71" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E72" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F72" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B73" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C73" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D73" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E73" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F73" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E74" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F74" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B75" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E75" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F75" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B76" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C76" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D76" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E76" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F76" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B77" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E77" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F77" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B78" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E78" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F78" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E79" t="s">
         <v>1</v>
@@ -1824,55 +1810,55 @@
     </row>
     <row r="80" spans="1:6" ht="51" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B80" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C80" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E80" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F80" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B81" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E81" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F81" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B82" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E82" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F82" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E83" t="s">
         <v>1</v>
@@ -1880,7 +1866,7 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E84" t="s">
         <v>1</v>
@@ -1888,84 +1874,84 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E85" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F85" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E86" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F86" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E87" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F87" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E88" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F88" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E89" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F89" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E90" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F90" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E91" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F91" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E92" t="s">
         <v>1</v>
@@ -1973,7 +1959,7 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E93" t="s">
         <v>1</v>
@@ -1981,7 +1967,7 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E94" t="s">
         <v>1</v>
@@ -1989,7 +1975,7 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E95" t="s">
         <v>1</v>
@@ -1997,7 +1983,7 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E96" t="s">
         <v>1</v>
@@ -2005,7 +1991,7 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E97" t="s">
         <v>1</v>
@@ -2013,7 +1999,7 @@
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E98" t="s">
         <v>1</v>
@@ -2021,10 +2007,10 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E99" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F99" t="s">
         <v>1</v>
@@ -2032,10 +2018,10 @@
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E100" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F100" t="s">
         <v>1</v>
@@ -2043,10 +2029,10 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E101" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F101" t="s">
         <v>1</v>
@@ -2054,10 +2040,10 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E102" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F102" t="s">
         <v>1</v>
@@ -2065,63 +2051,63 @@
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B103" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C103" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D103" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E103" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F103" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B104" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E104" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F104" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E105" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F105" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E106" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F106" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E107" t="s">
         <v>1</v>
@@ -2129,7 +2115,7 @@
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E108" t="s">
         <v>1</v>
@@ -2137,21 +2123,18 @@
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
-        <v>110</v>
-      </c>
-      <c r="B109" t="s">
-        <v>156</v>
+        <v>109</v>
       </c>
       <c r="E109" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F109" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E110" t="s">
         <v>1</v>
@@ -2159,21 +2142,18 @@
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
-        <v>112</v>
-      </c>
-      <c r="B111" t="s">
-        <v>157</v>
+        <v>111</v>
       </c>
       <c r="E111" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F111" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E112" t="s">
         <v>1</v>
@@ -2181,63 +2161,63 @@
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E113" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F113" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B114" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C114" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D114" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E114" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F114" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B115" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="E115" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F115" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E116" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F116" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E117" t="s">
         <v>1</v>
@@ -2245,7 +2225,7 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E118" t="s">
         <v>1</v>
@@ -2253,7 +2233,7 @@
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E119" t="s">
         <v>1</v>
@@ -2261,7 +2241,7 @@
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E120" t="s">
         <v>1</v>
@@ -2269,7 +2249,7 @@
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E121" t="s">
         <v>1</v>

</xml_diff>